<commit_message>
fix: standardize curve observation date
</commit_message>
<xml_diff>
--- a/outputs/019fdb9f-161f-7b22-9a01-b1a28036fbf3/capacity-source-register.xlsx
+++ b/outputs/019fdb9f-161f-7b22-9a01-b1a28036fbf3/capacity-source-register.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cutoff Policy" sheetId="1" r:id="R90413bd159994373"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Curve Inputs" sheetId="2" r:id="Rafda19bf871546af"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Register" sheetId="3" r:id="Ra984427b0ea84762"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cutoff Policy" sheetId="1" r:id="Rcb98fe5ae625438c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Curve Inputs" sheetId="2" r:id="Rae4c2eb312224165"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Register" sheetId="3" r:id="R39c3b30f53ba45cf"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -50,7 +50,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="5">
+  <x:fills count="8">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -72,6 +72,21 @@
         <x:fgColor rgb="FFF5F8FB"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17324D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17324D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17324D"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="1">
     <x:border/>
@@ -79,7 +94,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="28">
+  <x:cellXfs count="34">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -141,6 +156,20 @@
     </x:xf>
     <x:xf numFmtId="203" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -344,10 +373,10 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="31" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="43" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="64" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="3" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="25" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="35" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="18" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="18" hidden="0" customWidth="1"/>
@@ -356,23 +385,23 @@
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
       <x:c r="A1" s="3" t="str">
-        <x:v>Compute cost curve — dated evidence register</x:v>
+        <x:v>Compute cost curve — observation-date register</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="34" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>Two cutoffs keep the analysis honest: when the figure describes, and when the evidence became public.</x:v>
+        <x:v>The 31 December 2025 reference date governs displayed values. Publication timing is retained only as provenance.</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="42" customHeight="1">
       <x:c r="A4" s="8" t="str">
-        <x:v>Observation / effective-date cutoff</x:v>
+        <x:v>Observation reference date</x:v>
       </x:c>
       <x:c r="B4" s="9" t="n">
         <x:v>46022</x:v>
       </x:c>
       <x:c r="D4" s="12" t="str">
-        <x:v>Current curve audit</x:v>
+        <x:v>Headline observation audit</x:v>
       </x:c>
       <x:c r="E4" s="12" t="str">
         <x:v>Count</x:v>
@@ -380,13 +409,13 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="8" t="str">
-        <x:v>Research publication cutoff</x:v>
+        <x:v>Research publication cutoff (provenance note)</x:v>
       </x:c>
       <x:c r="B5" s="9" t="n">
         <x:v>46258</x:v>
       </x:c>
       <x:c r="D5" t="str">
-        <x:v>Bars in current chart</x:v>
+        <x:v>Records in current ledger</x:v>
       </x:c>
       <x:c r="E5" t="n">
         <x:f>COUNTA('Curve Inputs'!A5:A20)</x:f>
@@ -395,11 +424,11 @@
     </x:row>
     <x:row r="6">
       <x:c r="D6" t="str">
-        <x:v>Observation-aligned</x:v>
+        <x:v>Headline included</x:v>
       </x:c>
       <x:c r="E6" t="n">
-        <x:f>COUNTIF('Curve Inputs'!O5:O20,"Aligned")</x:f>
-        <x:v>14</x:v>
+        <x:f>COUNTIF('Curve Inputs'!R5:R20,"Included")</x:f>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="42" customHeight="1">
@@ -410,72 +439,72 @@
         <x:v>Treatment</x:v>
       </x:c>
       <x:c r="D7" t="str">
-        <x:v>Later than cutoff</x:v>
+        <x:v>Headline excluded</x:v>
       </x:c>
       <x:c r="E7" t="n">
+        <x:f>E5-E6</x:f>
+        <x:v>4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="14" t="str">
+        <x:v>Reference date</x:v>
+      </x:c>
+      <x:c r="B8" s="14" t="str">
+        <x:v>The headline uses the latest capacity observation and electricity-price period ending on or before 2025-12-31.</x:v>
+      </x:c>
+      <x:c r="D8" t="str">
+        <x:v>After reference date</x:v>
+      </x:c>
+      <x:c r="E8" t="n">
         <x:f>COUNTIF('Curve Inputs'!O5:O20,"Later than cutoff")</x:f>
         <x:v>1</x:v>
       </x:c>
     </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="14" t="str">
-        <x:v>Observation cutoff</x:v>
-      </x:c>
-      <x:c r="B8" s="14" t="str">
-        <x:v>The figure must describe a date or period ending on or before 2025-12-31.</x:v>
-      </x:c>
-      <x:c r="D8" t="str">
-        <x:v>Unknown observation date</x:v>
-      </x:c>
-      <x:c r="E8" t="n">
+    <x:row r="9">
+      <x:c r="A9" s="14" t="str">
+        <x:v>Exact source dates</x:v>
+      </x:c>
+      <x:c r="B9" s="14" t="str">
+        <x:v>Every input keeps its own observation or effective date visible so data age can be evaluated.</x:v>
+      </x:c>
+      <x:c r="D9" t="str">
+        <x:v>Unknown effective date</x:v>
+      </x:c>
+      <x:c r="E9" t="n">
         <x:f>COUNTIF('Curve Inputs'!O5:O20,"Unknown")</x:f>
         <x:v>1</x:v>
       </x:c>
     </x:row>
-    <x:row r="9">
-      <x:c r="A9" s="14" t="str">
-        <x:v>Publication cutoff</x:v>
-      </x:c>
-      <x:c r="B9" s="14" t="str">
-        <x:v>The source must have been public by 2026-08-24. Later publication of retrospective 2025 data is allowed.</x:v>
-      </x:c>
-      <x:c r="D9" t="str">
-        <x:v>Baseline-ready figures</x:v>
-      </x:c>
-      <x:c r="E9" t="n">
-        <x:f>COUNTIF('Source Register'!R5:R45,"Pass")</x:f>
-        <x:v>24</x:v>
-      </x:c>
-    </x:row>
     <x:row r="10">
       <x:c r="A10" s="14" t="str">
-        <x:v>Partial dates</x:v>
+        <x:v>Publication timing</x:v>
       </x:c>
       <x:c r="B10" s="14" t="str">
-        <x:v>Month, half-year, and year observations are normalized to period end and labelled with their precision.</x:v>
+        <x:v>Publication date is provenance only. It records when evidence became public but does not define the observation vintage.</x:v>
       </x:c>
       <x:c r="D10" t="str">
-        <x:v>Blank publication dates</x:v>
+        <x:v>Blank publication dates (note only)</x:v>
       </x:c>
       <x:c r="E10" t="n">
         <x:f>COUNTBLANK('Source Register'!J5:J45)</x:f>
-        <x:v>16</x:v>
+        <x:v>14</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="14" t="str">
-        <x:v>Targets / plans</x:v>
+        <x:v>Exclusions</x:v>
       </x:c>
       <x:c r="B11" s="14" t="str">
-        <x:v>Kept in the register but not treated as observed capacity or realised price.</x:v>
+        <x:v>Targets, post-2025 values, prices with no effective date, and unsupported source matches are not plotted.</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="14" t="str">
-        <x:v>Unknown publication dates</x:v>
+        <x:v>Partial dates</x:v>
       </x:c>
       <x:c r="B12" s="14" t="str">
-        <x:v>Recorded as unknown. They do not silently pass the publication test.</x:v>
+        <x:v>Month, half-year, and year observations are normalized to period end and labelled with their precision.</x:v>
       </x:c>
       <x:c r="D12" s="10" t="str">
         <x:v>Interpretation</x:v>
@@ -487,10 +516,10 @@
     </x:row>
     <x:row r="13">
       <x:c r="D13" s="16" t="str">
-        <x:v>Aligned</x:v>
+        <x:v>Included</x:v>
       </x:c>
       <x:c r="E13" s="14" t="str">
-        <x:v>Both the capacity observation and electricity-price effective date are no later than the observation cutoff.</x:v>
+        <x:v>Latest observed/effective input ends on or before the reference date and is not a target.</x:v>
       </x:c>
       <x:c r="F13" s="14"/>
       <x:c r="G13" s="14"/>
@@ -498,10 +527,10 @@
     </x:row>
     <x:row r="14">
       <x:c r="D14" s="16" t="str">
-        <x:v>Later than cutoff</x:v>
+        <x:v>Excluded</x:v>
       </x:c>
       <x:c r="E14" s="14" t="str">
-        <x:v>At least one current input describes a date after the observation cutoff.</x:v>
+        <x:v>A target, post-reference value, undated effective price, or unsupported source match is kept in the ledger but not plotted.</x:v>
       </x:c>
       <x:c r="F14" s="14"/>
       <x:c r="G14" s="14"/>
@@ -509,10 +538,10 @@
     </x:row>
     <x:row r="15">
       <x:c r="D15" s="16" t="str">
-        <x:v>Unknown</x:v>
+        <x:v>Exact dates</x:v>
       </x:c>
       <x:c r="E15" s="14" t="str">
-        <x:v>At least one observation/effective date is missing, so alignment cannot be established.</x:v>
+        <x:v>The reference-date rule does not claim that every source was measured on the same day; source dates remain visible.</x:v>
       </x:c>
       <x:c r="F15" s="14"/>
       <x:c r="G15" s="14"/>
@@ -520,10 +549,10 @@
     </x:row>
     <x:row r="16">
       <x:c r="D16" s="16" t="str">
-        <x:v>Publication flag</x:v>
+        <x:v>Publication note</x:v>
       </x:c>
       <x:c r="E16" s="14" t="str">
-        <x:v>A separate flag shows whether the evidence was public by the research cutoff.</x:v>
+        <x:v>24 August 2026 records when research was frozen. It does not control the plotted vintage.</x:v>
       </x:c>
       <x:c r="F16" s="14"/>
       <x:c r="G16" s="14"/>
@@ -564,69 +593,73 @@
     <x:col min="15" max="15" width="18" hidden="0" customWidth="1"/>
     <x:col min="16" max="16" width="42" hidden="0" customWidth="1"/>
     <x:col min="17" max="17" width="72" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="27" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
       <x:c r="A1" s="3" t="str">
-        <x:v>Current chart inputs</x:v>
+        <x:v>Current chart inputs — observation-date decisions</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="34" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>This is the exact width-and-height dataset currently used by the published chart, audited against the two cutoffs.</x:v>
+        <x:v>Observation timing governs the headline. Publication dates are shown only to document provenance.</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="42" customHeight="1">
-      <x:c r="A4" s="12" t="str">
+      <x:c r="A4" s="33" t="str">
         <x:v>Bar ID</x:v>
       </x:c>
-      <x:c r="B4" s="12" t="str">
+      <x:c r="B4" s="33" t="str">
         <x:v>Country</x:v>
       </x:c>
-      <x:c r="C4" s="12" t="str">
+      <x:c r="C4" s="33" t="str">
         <x:v>Location</x:v>
       </x:c>
-      <x:c r="D4" s="12" t="str">
+      <x:c r="D4" s="33" t="str">
         <x:v>Capacity (MW)</x:v>
       </x:c>
-      <x:c r="E4" s="12" t="str">
+      <x:c r="E4" s="33" t="str">
         <x:v>Capacity as of</x:v>
       </x:c>
-      <x:c r="F4" s="12" t="str">
+      <x:c r="F4" s="33" t="str">
         <x:v>Capacity published</x:v>
       </x:c>
-      <x:c r="G4" s="12" t="str">
+      <x:c r="G4" s="33" t="str">
         <x:v>Capacity ≤ cutoff?</x:v>
       </x:c>
-      <x:c r="H4" s="12" t="str">
+      <x:c r="H4" s="33" t="str">
         <x:v>Electricity (USD/kWh)</x:v>
       </x:c>
-      <x:c r="I4" s="12" t="str">
+      <x:c r="I4" s="33" t="str">
         <x:v>Price effective</x:v>
       </x:c>
-      <x:c r="J4" s="12" t="str">
+      <x:c r="J4" s="33" t="str">
         <x:v>Price published</x:v>
       </x:c>
-      <x:c r="K4" s="12" t="str">
+      <x:c r="K4" s="33" t="str">
         <x:v>Price ≤ cutoff?</x:v>
       </x:c>
-      <x:c r="L4" s="12" t="str">
+      <x:c r="L4" s="33" t="str">
         <x:v>Capacity source known?</x:v>
       </x:c>
-      <x:c r="M4" s="12" t="str">
+      <x:c r="M4" s="33" t="str">
         <x:v>Price source known?</x:v>
       </x:c>
-      <x:c r="N4" s="12" t="str">
-        <x:v>Publication status</x:v>
-      </x:c>
-      <x:c r="O4" s="12" t="str">
+      <x:c r="N4" s="33" t="str">
+        <x:v>Publication note</x:v>
+      </x:c>
+      <x:c r="O4" s="33" t="str">
         <x:v>Observation status</x:v>
       </x:c>
-      <x:c r="P4" s="12" t="str">
+      <x:c r="P4" s="33" t="str">
         <x:v>Capacity source</x:v>
       </x:c>
-      <x:c r="Q4" s="12" t="str">
+      <x:c r="Q4" s="33" t="str">
         <x:v>Price source / notes</x:v>
+      </x:c>
+      <x:c r="R4" s="33" t="str">
+        <x:v>Headline decision</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -687,6 +720,9 @@
       <x:c r="Q5" s="14" t="str">
         <x:v>https://www.nea.gov.cn/20250718/410e42d872e4417687cb5b0ab357d088/c.html — Documented 11-centre subset; capacity derived as 326 MW facility power / PUE 1.21.</x:v>
       </x:c>
+      <x:c r="R5" s="14" t="str">
+        <x:v>Included</x:v>
+      </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="14" t="str">
@@ -746,6 +782,9 @@
       <x:c r="Q6" s="14" t="str">
         <x:v>https://nyj.guizhou.gov.cn/zwgk/xxgkml/zdlyxx/czzj/202503/P020250307503578350701.pdf — Capacity derived from 137,400 powered-on standard racks at 2.5 kW; price is a 2025 policy target.</x:v>
       </x:c>
+      <x:c r="R6" s="14" t="str">
+        <x:v>Excluded: target price</x:v>
+      </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="14" t="str">
@@ -804,6 +843,9 @@
       </x:c>
       <x:c r="Q7" s="14" t="str">
         <x:v>https://www.xlgl.gov.cn/xlgl/zw/zwgk/tzgg/2025090509233740836/index.html — Provincial treemap estimate less the Hohhot subset; price is a tariff proxy at 90% load factor.</x:v>
+      </x:c>
+      <x:c r="R7" s="14" t="str">
+        <x:v>Included</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -862,6 +904,9 @@
       <x:c r="Q8" s="14" t="str">
         <x:v>https://energydc.cn/policy/sx/2026-04/cbe2e026-2c0e-11f1-9e60-f679c2336431 — Capacity is a treemap estimate. Price uses an April 2026 secondary tariff page; exact publication day not recorded.</x:v>
       </x:c>
+      <x:c r="R8" s="14" t="str">
+        <x:v>Excluded: post-2025 price</x:v>
+      </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="14" t="str">
@@ -919,6 +964,9 @@
       <x:c r="Q9" s="14" t="str">
         <x:v>https://zjjcmspublic.oss-cn-hangzhou-zwynet-d01-a.internet.cloud.zj.gov.cn/jcms_files/jcms1/web2241/site/attach/0/d94d1693bc7042f0a4349368bbb18419.pdf — Capacity is a treemap estimate. June 2025 tariff attachment has no recorded webpage publication date.</x:v>
       </x:c>
+      <x:c r="R9" s="14" t="str">
+        <x:v>Included</x:v>
+      </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="14" t="str">
@@ -978,6 +1026,9 @@
       <x:c r="Q10" s="14" t="str">
         <x:v>https://www.lp.gov.cn/newsite/xwdt/gsgg_5768869/202505/P020250530625753057568.pdf — Provincial treemap estimate less Gui'an; price is a tariff proxy at 90% load factor.</x:v>
       </x:c>
+      <x:c r="R10" s="14" t="str">
+        <x:v>Included</x:v>
+      </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="14" t="str">
@@ -1035,6 +1086,9 @@
       <x:c r="Q11" s="14" t="str">
         <x:v>https://ele.aiit.org.cn/static/elefile/99303281758074622710101893155890.pdf — Capacity is a treemap estimate; Jibei tariff proxy used for the province. Publication day for tariff PDF is unrecorded.</x:v>
       </x:c>
+      <x:c r="R11" s="14" t="str">
+        <x:v>Included</x:v>
+      </x:c>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="14" t="str">
@@ -1094,6 +1148,9 @@
       <x:c r="Q12" s="14" t="str">
         <x:v>https://www.jintan.gov.cn/html/czjt/2025/JFKEQAOD_0624/281022.html — Capacity is a treemap estimate; price is a tariff proxy at 90% load factor.</x:v>
       </x:c>
+      <x:c r="R12" s="14" t="str">
+        <x:v>Included</x:v>
+      </x:c>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="14" t="str">
@@ -1151,6 +1208,9 @@
       <x:c r="Q13" s="14" t="str">
         <x:v>https://ele.aiit.org.cn/static/elefile/99303281924019507384201247156397.pdf — Capacity is a treemap estimate. Publication day for tariff PDF is unrecorded.</x:v>
       </x:c>
+      <x:c r="R13" s="14" t="str">
+        <x:v>Included</x:v>
+      </x:c>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="14" t="str">
@@ -1208,6 +1268,9 @@
       <x:c r="Q14" s="14" t="str">
         <x:v>https://www.gdsx.gov.cn/sgsxgdj/attachment/0/272/272080/2734391.pdf — Capacity is a treemap estimate; price is a capacity-weighted northern Guangdong / Pearl River proxy.</x:v>
       </x:c>
+      <x:c r="R14" s="14" t="str">
+        <x:v>Included</x:v>
+      </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="14" t="str">
@@ -1267,6 +1330,9 @@
       <x:c r="Q15" s="14" t="str">
         <x:v>https://www.yantai.gov.cn/art/2025/3/20/art_70253_3244147.html — Capacity is a treemap estimate; price is a tariff proxy at 90% load factor.</x:v>
       </x:c>
+      <x:c r="R15" s="14" t="str">
+        <x:v>Included</x:v>
+      </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="14" t="str">
@@ -1324,6 +1390,9 @@
       <x:c r="Q16" s="14" t="str">
         <x:v>https://www.shanghai.gov.cn/cmsres/8d/8dbc9d8c392e43b791295f493f1d247e/5b1658885ab19ab927050e05dfbb83f9.pdf — Capacity is a treemap estimate. The linked tariff source needs replacement: it appears to be a policy notice, not the June tariff table.</x:v>
       </x:c>
+      <x:c r="R16" s="14" t="str">
+        <x:v>Excluded: source mismatch</x:v>
+      </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="14" t="str">
@@ -1380,6 +1449,9 @@
       </x:c>
       <x:c r="Q17" s="14" t="str">
         <x:v>https://www.hydroquebec.com/data/documents-donnees/pdf/rates-chart-2025.pdf — Wholesale H2 2025 market inventory; Rate L effective price. Rate-chart publication day is unrecorded.</x:v>
+      </x:c>
+      <x:c r="R17" s="14" t="str">
+        <x:v>Included</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -1436,6 +1508,9 @@
       <x:c r="Q18" s="14" t="str">
         <x:v>https://sera.gov.sa/en/consumer/electric-tariff/electric-tariff-categories/consumption-tariff — National operating capacity; regulated cloud tariff page is undated/current.</x:v>
       </x:c>
+      <x:c r="R18" s="14" t="str">
+        <x:v>Excluded: price date unknown</x:v>
+      </x:c>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="14" t="str">
@@ -1461,12 +1536,14 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="H19" s="24" t="n">
-        <x:v>0.0612</x:v>
+        <x:v>0.0655</x:v>
       </x:c>
       <x:c r="I19" s="23" t="n">
-        <x:v>45657</x:v>
-      </x:c>
-      <x:c r="J19" s="23"/>
+        <x:v>46022</x:v>
+      </x:c>
+      <x:c r="J19" s="23" t="n">
+        <x:v>46073</x:v>
+      </x:c>
       <x:c r="K19" s="14" t="str">
         <x:f>IF(I19="","Unknown",IF(I19&lt;='Cutoff Policy'!$B$4,"Yes","No"))</x:f>
         <x:v>Yes</x:v>
@@ -1477,11 +1554,11 @@
       </x:c>
       <x:c r="M19" s="14" t="str">
         <x:f>IF(J19="","Unknown",IF(J19&lt;='Cutoff Policy'!$B$5,"Yes","No"))</x:f>
-        <x:v>Unknown</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N19" s="14" t="str">
         <x:f>IF(OR(L19="Unknown",M19="Unknown"),"Incomplete date record",IF(AND(L19="Yes",M19="Yes"),"Pass","After research cutoff"))</x:f>
-        <x:v>Incomplete date record</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="O19" s="14" t="str">
         <x:f>IF(OR(G19="Unknown",K19="Unknown"),"Unknown",IF(AND(G19="Yes",K19="Yes"),"Aligned","Later than cutoff"))</x:f>
@@ -1491,7 +1568,10 @@
         <x:v>https://www.cbre.com/press-releases/northern-virginia-extends-lead-as-largest-u-s-data-center-market-in-2025</x:v>
       </x:c>
       <x:c r="Q19" s="14" t="str">
-        <x:v>https://www.eia.gov/electricity/annual/table.php?t=epa_02_10.html — Wholesale H2 2025 market inventory; 2024 Texas industrial average, not a hyperscale contract.</x:v>
+        <x:v>https://www.eia.gov/electricity/monthly/current_month/february2026.pdf — EIA table 5.6.B preliminary calendar-2025 Texas industrial average: 6.55 cents/kWh.</x:v>
+      </x:c>
+      <x:c r="R19" s="14" t="str">
+        <x:v>Included</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
@@ -1518,12 +1598,14 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="H20" s="24" t="n">
-        <x:v>0.0899</x:v>
+        <x:v>0.0945</x:v>
       </x:c>
       <x:c r="I20" s="23" t="n">
-        <x:v>45657</x:v>
-      </x:c>
-      <x:c r="J20" s="23"/>
+        <x:v>46022</x:v>
+      </x:c>
+      <x:c r="J20" s="23" t="n">
+        <x:v>46073</x:v>
+      </x:c>
       <x:c r="K20" s="14" t="str">
         <x:f>IF(I20="","Unknown",IF(I20&lt;='Cutoff Policy'!$B$4,"Yes","No"))</x:f>
         <x:v>Yes</x:v>
@@ -1534,11 +1616,11 @@
       </x:c>
       <x:c r="M20" s="14" t="str">
         <x:f>IF(J20="","Unknown",IF(J20&lt;='Cutoff Policy'!$B$5,"Yes","No"))</x:f>
-        <x:v>Unknown</x:v>
+        <x:v>Yes</x:v>
       </x:c>
       <x:c r="N20" s="14" t="str">
         <x:f>IF(OR(L20="Unknown",M20="Unknown"),"Incomplete date record",IF(AND(L20="Yes",M20="Yes"),"Pass","After research cutoff"))</x:f>
-        <x:v>Incomplete date record</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="O20" s="14" t="str">
         <x:f>IF(OR(G20="Unknown",K20="Unknown"),"Unknown",IF(AND(G20="Yes",K20="Yes"),"Aligned","Later than cutoff"))</x:f>
@@ -1548,13 +1630,16 @@
         <x:v>https://www.cbre.com/press-releases/northern-virginia-extends-lead-as-largest-u-s-data-center-market-in-2025</x:v>
       </x:c>
       <x:c r="Q20" s="14" t="str">
-        <x:v>https://www.eia.gov/electricity/annual/table.php?t=epa_02_10.html — Wholesale H2 2025 market inventory; 2024 Virginia industrial average, not a hyperscale contract.</x:v>
+        <x:v>https://www.eia.gov/electricity/monthly/current_month/february2026.pdf — EIA table 5.6.B preliminary calendar-2025 Virginia industrial average: 9.45 cents/kWh.</x:v>
+      </x:c>
+      <x:c r="R20" s="14" t="str">
+        <x:v>Included</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:Q1"/>
-    <x:mergeCell ref="A2:Q2"/>
+    <x:mergeCell ref="A1:R1"/>
+    <x:mergeCell ref="A2:R2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -1592,7 +1677,7 @@
     </x:row>
     <x:row r="2" ht="34" customHeight="1">
       <x:c r="A2" s="7" t="str">
-        <x:v>One row per sourced or derived figure. Blank publication dates are deliberate: the source is undated or the exact release day has not yet been established.</x:v>
+        <x:v>Observation/effective dates determine eligibility. Publication dates remain in the register as provenance only.</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="42" customHeight="1">
@@ -1645,10 +1730,10 @@
         <x:v>Observation cutoff</x:v>
       </x:c>
       <x:c r="Q4" s="12" t="str">
-        <x:v>Publication cutoff</x:v>
+        <x:v>Publication note only</x:v>
       </x:c>
       <x:c r="R4" s="12" t="str">
-        <x:v>Overall status</x:v>
+        <x:v>Observation eligibility</x:v>
       </x:c>
       <x:c r="S4" s="12" t="str">
         <x:v>Boundary / notes</x:v>
@@ -1709,8 +1794,8 @@
         <x:v>Pass</x:v>
       </x:c>
       <x:c r="R5" s="14" t="str">
-        <x:f>IF(OR(P5="After cutoff",Q5="After cutoff"),"Exclude from baseline",IF(OR(P5="Unknown",Q5="Unknown"),"Needs date / judgment",IF(G5="Target","Target only","Pass")))</x:f>
-        <x:v>Pass</x:v>
+        <x:f>IF(P5="After cutoff","Exclude: post-reference",IF(P5="Unknown","Needs observation date",IF(G5="Target","Target only","Observation-eligible")))</x:f>
+        <x:v>Observation-eligible</x:v>
       </x:c>
       <x:c r="S5" s="14" t="str">
         <x:v>Official national total; in-use standard racks.</x:v>
@@ -1771,8 +1856,8 @@
         <x:v>Pass</x:v>
       </x:c>
       <x:c r="R6" s="14" t="str">
-        <x:f>IF(OR(P6="After cutoff",Q6="After cutoff"),"Exclude from baseline",IF(OR(P6="Unknown",Q6="Unknown"),"Needs date / judgment",IF(G6="Target","Target only","Pass")))</x:f>
-        <x:v>Pass</x:v>
+        <x:f>IF(P6="After cutoff","Exclude: post-reference",IF(P6="Unknown","Needs observation date",IF(G6="Target","Target only","Observation-eligible")))</x:f>
+        <x:v>Observation-eligible</x:v>
       </x:c>
       <x:c r="S6" s="14" t="str">
         <x:v>The report publishes a treemap, not a numeric table; figures are estimates derived from rectangle areas.</x:v>
@@ -1833,8 +1918,8 @@
         <x:v>Pass</x:v>
       </x:c>
       <x:c r="R7" s="14" t="str">
-        <x:f>IF(OR(P7="After cutoff",Q7="After cutoff"),"Exclude from baseline",IF(OR(P7="Unknown",Q7="Unknown"),"Needs date / judgment",IF(G7="Target","Target only","Pass")))</x:f>
-        <x:v>Pass</x:v>
+        <x:f>IF(P7="After cutoff","Exclude: post-reference",IF(P7="Unknown","Needs observation date",IF(G7="Target","Target only","Observation-eligible")))</x:f>
+        <x:v>Observation-eligible</x:v>
       </x:c>
       <x:c r="S7" s="14" t="str">
         <x:v>Underlying figure for the 269.4 MW IT-capacity subset.</x:v>
@@ -1895,8 +1980,8 @@
         <x:v>Pass</x:v>
       </x:c>
       <x:c r="R8" s="14" t="str">
-        <x:f>IF(OR(P8="After cutoff",Q8="After cutoff"),"Exclude from baseline",IF(OR(P8="Unknown",Q8="Unknown"),"Needs date / judgment",IF(G8="Target","Target only","Pass")))</x:f>
-        <x:v>Pass</x:v>
+        <x:f>IF(P8="After cutoff","Exclude: post-reference",IF(P8="Unknown","Needs observation date",IF(G8="Target","Target only","Observation-eligible")))</x:f>
+        <x:v>Observation-eligible</x:v>
       </x:c>
       <x:c r="S8" s="14" t="str">
         <x:v>Used only to convert the documented subset's facility MW to IT MW.</x:v>
@@ -1957,8 +2042,8 @@
         <x:v>Pass</x:v>
       </x:c>
       <x:c r="R9" s="14" t="str">
-        <x:f>IF(OR(P9="After cutoff",Q9="After cutoff"),"Exclude from baseline",IF(OR(P9="Unknown",Q9="Unknown"),"Needs date / judgment",IF(G9="Target","Target only","Pass")))</x:f>
-        <x:v>Pass</x:v>
+        <x:f>IF(P9="After cutoff","Exclude: post-reference",IF(P9="Unknown","Needs observation date",IF(G9="Target","Target only","Observation-eligible")))</x:f>
+        <x:v>Observation-eligible</x:v>
       </x:c>
       <x:c r="S9" s="14" t="str">
         <x:v>Converted at the CAICT standard-rack basis of 2.5 kW.</x:v>
@@ -2019,8 +2104,8 @@
         <x:v>Pass</x:v>
       </x:c>
       <x:c r="R10" s="14" t="str">
-        <x:f>IF(OR(P10="After cutoff",Q10="After cutoff"),"Exclude from baseline",IF(OR(P10="Unknown",Q10="Unknown"),"Needs date / judgment",IF(G10="Target","Target only","Pass")))</x:f>
-        <x:v>Pass</x:v>
+        <x:f>IF(P10="After cutoff","Exclude: post-reference",IF(P10="Unknown","Needs observation date",IF(G10="Target","Target only","Observation-eligible")))</x:f>
+        <x:v>Observation-eligible</x:v>
       </x:c>
       <x:c r="S10" s="14" t="str">
         <x:v>Article reports the local transaction price; no separate measurement date stated.</x:v>
@@ -2070,7 +2155,7 @@
         <x:v>https://nyj.guizhou.gov.cn/zwgk/xxgkml/zdlyxx/czzj/202503/P020250307503578350701.pdf</x:v>
       </x:c>
       <x:c r="O11" s="14" t="str">
-        <x:v>Yes – chart height</x:v>
+        <x:v>No — excluded target</x:v>
       </x:c>
       <x:c r="P11" s="14" t="str">
         <x:f>IF(H11="","Unknown",IF(H11&lt;='Cutoff Policy'!$B$4,"Pass","After cutoff"))</x:f>
@@ -2081,7 +2166,7 @@
         <x:v>Pass</x:v>
       </x:c>
       <x:c r="R11" s="14" t="str">
-        <x:f>IF(OR(P11="After cutoff",Q11="After cutoff"),"Exclude from baseline",IF(OR(P11="Unknown",Q11="Unknown"),"Needs date / judgment",IF(G11="Target","Target only","Pass")))</x:f>
+        <x:f>IF(P11="After cutoff","Exclude: post-reference",IF(P11="Unknown","Needs observation date",IF(G11="Target","Target only","Observation-eligible")))</x:f>
         <x:v>Target only</x:v>
       </x:c>
       <x:c r="S11" s="14" t="str">
@@ -2143,8 +2228,8 @@
         <x:v>Pass</x:v>
       </x:c>
       <x:c r="R12" s="14" t="str">
-        <x:f>IF(OR(P12="After cutoff",Q12="After cutoff"),"Exclude from baseline",IF(OR(P12="Unknown",Q12="Unknown"),"Needs date / judgment",IF(G12="Target","Target only","Pass")))</x:f>
-        <x:v>Pass</x:v>
+        <x:f>IF(P12="After cutoff","Exclude: post-reference",IF(P12="Unknown","Needs observation date",IF(G12="Target","Target only","Observation-eligible")))</x:f>
+        <x:v>Observation-eligible</x:v>
       </x:c>
       <x:c r="S12" s="14" t="str">
         <x:v>Energy charge plus maximum-demand charge spread over 730 hours at 90% load factor.</x:v>
@@ -2192,7 +2277,7 @@
         <x:v>https://energydc.cn/policy/sx/2026-04/cbe2e026-2c0e-11f1-9e60-f679c2336431</x:v>
       </x:c>
       <x:c r="O13" s="14" t="str">
-        <x:v>Yes – chart height</x:v>
+        <x:v>No — excluded post-2025</x:v>
       </x:c>
       <x:c r="P13" s="14" t="str">
         <x:f>IF(H13="","Unknown",IF(H13&lt;='Cutoff Policy'!$B$4,"Pass","After cutoff"))</x:f>
@@ -2203,8 +2288,8 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="R13" s="14" t="str">
-        <x:f>IF(OR(P13="After cutoff",Q13="After cutoff"),"Exclude from baseline",IF(OR(P13="Unknown",Q13="Unknown"),"Needs date / judgment",IF(G13="Target","Target only","Pass")))</x:f>
-        <x:v>Exclude from baseline</x:v>
+        <x:f>IF(P13="After cutoff","Exclude: post-reference",IF(P13="Unknown","Needs observation date",IF(G13="Target","Target only","Observation-eligible")))</x:f>
+        <x:v>Exclude: post-reference</x:v>
       </x:c>
       <x:c r="S13" s="14" t="str">
         <x:v>Fails the end-2025 observation cutoff and is a secondary source.</x:v>
@@ -2263,8 +2348,8 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="R14" s="14" t="str">
-        <x:f>IF(OR(P14="After cutoff",Q14="After cutoff"),"Exclude from baseline",IF(OR(P14="Unknown",Q14="Unknown"),"Needs date / judgment",IF(G14="Target","Target only","Pass")))</x:f>
-        <x:v>Needs date / judgment</x:v>
+        <x:f>IF(P14="After cutoff","Exclude: post-reference",IF(P14="Unknown","Needs observation date",IF(G14="Target","Target only","Observation-eligible")))</x:f>
+        <x:v>Observation-eligible</x:v>
       </x:c>
       <x:c r="S14" s="14" t="str">
         <x:v>Official attachment; publication day still needs a landing-page record.</x:v>
@@ -2325,8 +2410,8 @@
         <x:v>Pass</x:v>
       </x:c>
       <x:c r="R15" s="14" t="str">
-        <x:f>IF(OR(P15="After cutoff",Q15="After cutoff"),"Exclude from baseline",IF(OR(P15="Unknown",Q15="Unknown"),"Needs date / judgment",IF(G15="Target","Target only","Pass")))</x:f>
-        <x:v>Pass</x:v>
+        <x:f>IF(P15="After cutoff","Exclude: post-reference",IF(P15="Unknown","Needs observation date",IF(G15="Target","Target only","Observation-eligible")))</x:f>
+        <x:v>Observation-eligible</x:v>
       </x:c>
       <x:c r="S15" s="14" t="str">
         <x:v>Energy charge plus demand charge at 90% load factor.</x:v>
@@ -2385,8 +2470,8 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="R16" s="14" t="str">
-        <x:f>IF(OR(P16="After cutoff",Q16="After cutoff"),"Exclude from baseline",IF(OR(P16="Unknown",Q16="Unknown"),"Needs date / judgment",IF(G16="Target","Target only","Pass")))</x:f>
-        <x:v>Needs date / judgment</x:v>
+        <x:f>IF(P16="After cutoff","Exclude: post-reference",IF(P16="Unknown","Needs observation date",IF(G16="Target","Target only","Observation-eligible")))</x:f>
+        <x:v>Observation-eligible</x:v>
       </x:c>
       <x:c r="S16" s="14" t="str">
         <x:v>Official tariff PDF; exact webpage publication date is not recorded.</x:v>
@@ -2447,8 +2532,8 @@
         <x:v>Pass</x:v>
       </x:c>
       <x:c r="R17" s="14" t="str">
-        <x:f>IF(OR(P17="After cutoff",Q17="After cutoff"),"Exclude from baseline",IF(OR(P17="Unknown",Q17="Unknown"),"Needs date / judgment",IF(G17="Target","Target only","Pass")))</x:f>
-        <x:v>Pass</x:v>
+        <x:f>IF(P17="After cutoff","Exclude: post-reference",IF(P17="Unknown","Needs observation date",IF(G17="Target","Target only","Observation-eligible")))</x:f>
+        <x:v>Observation-eligible</x:v>
       </x:c>
       <x:c r="S17" s="14" t="str">
         <x:v>Energy charge plus demand charge at 90% load factor.</x:v>
@@ -2507,8 +2592,8 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="R18" s="14" t="str">
-        <x:f>IF(OR(P18="After cutoff",Q18="After cutoff"),"Exclude from baseline",IF(OR(P18="Unknown",Q18="Unknown"),"Needs date / judgment",IF(G18="Target","Target only","Pass")))</x:f>
-        <x:v>Needs date / judgment</x:v>
+        <x:f>IF(P18="After cutoff","Exclude: post-reference",IF(P18="Unknown","Needs observation date",IF(G18="Target","Target only","Observation-eligible")))</x:f>
+        <x:v>Observation-eligible</x:v>
       </x:c>
       <x:c r="S18" s="14" t="str">
         <x:v>Official tariff PDF; exact webpage publication date is not recorded.</x:v>
@@ -2567,8 +2652,8 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="R19" s="14" t="str">
-        <x:f>IF(OR(P19="After cutoff",Q19="After cutoff"),"Exclude from baseline",IF(OR(P19="Unknown",Q19="Unknown"),"Needs date / judgment",IF(G19="Target","Target only","Pass")))</x:f>
-        <x:v>Needs date / judgment</x:v>
+        <x:f>IF(P19="After cutoff","Exclude: post-reference",IF(P19="Unknown","Needs observation date",IF(G19="Target","Target only","Observation-eligible")))</x:f>
+        <x:v>Observation-eligible</x:v>
       </x:c>
       <x:c r="S19" s="14" t="str">
         <x:v>Weighted between northern Guangdong and Pearl River Delta proxies.</x:v>
@@ -2629,8 +2714,8 @@
         <x:v>Pass</x:v>
       </x:c>
       <x:c r="R20" s="14" t="str">
-        <x:f>IF(OR(P20="After cutoff",Q20="After cutoff"),"Exclude from baseline",IF(OR(P20="Unknown",Q20="Unknown"),"Needs date / judgment",IF(G20="Target","Target only","Pass")))</x:f>
-        <x:v>Pass</x:v>
+        <x:f>IF(P20="After cutoff","Exclude: post-reference",IF(P20="Unknown","Needs observation date",IF(G20="Target","Target only","Observation-eligible")))</x:f>
+        <x:v>Observation-eligible</x:v>
       </x:c>
       <x:c r="S20" s="14" t="str">
         <x:v>Energy charge plus demand charge at 90% load factor.</x:v>
@@ -2678,7 +2763,7 @@
         <x:v>https://www.shanghai.gov.cn/cmsres/8d/8dbc9d8c392e43b791295f493f1d247e/5b1658885ab19ab927050e05dfbb83f9.pdf</x:v>
       </x:c>
       <x:c r="O21" s="14" t="str">
-        <x:v>Yes – chart height</x:v>
+        <x:v>No — excluded source mismatch</x:v>
       </x:c>
       <x:c r="P21" s="14" t="str">
         <x:f>IF(H21="","Unknown",IF(H21&lt;='Cutoff Policy'!$B$4,"Pass","After cutoff"))</x:f>
@@ -2689,8 +2774,7 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="R21" s="14" t="str">
-        <x:f>IF(OR(P21="After cutoff",Q21="After cutoff"),"Exclude from baseline",IF(OR(P21="Unknown",Q21="Unknown"),"Needs date / judgment",IF(G21="Target","Target only","Pass")))</x:f>
-        <x:v>Needs date / judgment</x:v>
+        <x:v>Exclude: source mismatch</x:v>
       </x:c>
       <x:c r="S21" s="14" t="str">
         <x:v>Needs replacement: linked document does not clearly establish the claimed June 2025 proxy.</x:v>
@@ -2749,8 +2833,8 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="R22" s="14" t="str">
-        <x:f>IF(OR(P22="After cutoff",Q22="After cutoff"),"Exclude from baseline",IF(OR(P22="Unknown",Q22="Unknown"),"Needs date / judgment",IF(G22="Target","Target only","Pass")))</x:f>
-        <x:v>Needs date / judgment</x:v>
+        <x:f>IF(P22="After cutoff","Exclude: post-reference",IF(P22="Unknown","Needs observation date",IF(G22="Target","Target only","Observation-eligible")))</x:f>
+        <x:v>Observation-eligible</x:v>
       </x:c>
       <x:c r="S22" s="14" t="str">
         <x:v>Effective price at 120 kV and 100% load factor.</x:v>
@@ -2796,7 +2880,7 @@
         <x:v>https://sera.gov.sa/en/consumer/electric-tariff/electric-tariff-categories/consumption-tariff</x:v>
       </x:c>
       <x:c r="O23" s="14" t="str">
-        <x:v>Yes – chart height</x:v>
+        <x:v>No — excluded date unknown</x:v>
       </x:c>
       <x:c r="P23" s="14" t="str">
         <x:f>IF(H23="","Unknown",IF(H23&lt;='Cutoff Policy'!$B$4,"Pass","After cutoff"))</x:f>
@@ -2807,8 +2891,8 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="R23" s="14" t="str">
-        <x:f>IF(OR(P23="After cutoff",Q23="After cutoff"),"Exclude from baseline",IF(OR(P23="Unknown",Q23="Unknown"),"Needs date / judgment",IF(G23="Target","Target only","Pass")))</x:f>
-        <x:v>Needs date / judgment</x:v>
+        <x:f>IF(P23="After cutoff","Exclude: post-reference",IF(P23="Unknown","Needs observation date",IF(G23="Target","Target only","Observation-eligible")))</x:f>
+        <x:v>Needs observation date</x:v>
       </x:c>
       <x:c r="S23" s="14" t="str">
         <x:v>Current webpage is undated; archival effective date is still needed.</x:v>
@@ -2828,7 +2912,7 @@
         <x:v>Texas</x:v>
       </x:c>
       <x:c r="E24" s="27" t="n">
-        <x:v>0.0612</x:v>
+        <x:v>0.0655</x:v>
       </x:c>
       <x:c r="F24" s="14" t="str">
         <x:v>USD/kWh</x:v>
@@ -2837,23 +2921,25 @@
         <x:v>Reported average</x:v>
       </x:c>
       <x:c r="H24" s="23" t="n">
-        <x:v>45657</x:v>
+        <x:v>46022</x:v>
       </x:c>
       <x:c r="I24" s="14" t="str">
         <x:v>Calendar year end</x:v>
       </x:c>
-      <x:c r="J24" s="23"/>
+      <x:c r="J24" s="23" t="n">
+        <x:v>46073</x:v>
+      </x:c>
       <x:c r="K24" s="14" t="str">
-        <x:v>Release day unrecorded</x:v>
+        <x:v>EIA preliminary release</x:v>
       </x:c>
       <x:c r="L24" s="14" t="str">
         <x:v>U.S. Energy Information Administration</x:v>
       </x:c>
       <x:c r="M24" s="14" t="str">
-        <x:v>Electric Power Annual table 2.10</x:v>
+        <x:v>Electric Power Monthly table 5.6.B</x:v>
       </x:c>
       <x:c r="N24" s="14" t="str">
-        <x:v>https://www.eia.gov/electricity/annual/table.php?t=epa_02_10.html</x:v>
+        <x:v>https://www.eia.gov/electricity/monthly/current_month/february2026.pdf</x:v>
       </x:c>
       <x:c r="O24" s="14" t="str">
         <x:v>Yes – chart height</x:v>
@@ -2864,14 +2950,14 @@
       </x:c>
       <x:c r="Q24" s="14" t="str">
         <x:f>IF(J24="","Unknown",IF(J24&lt;='Cutoff Policy'!$B$5,"Pass","After cutoff"))</x:f>
-        <x:v>Unknown</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="R24" s="14" t="str">
-        <x:f>IF(OR(P24="After cutoff",Q24="After cutoff"),"Exclude from baseline",IF(OR(P24="Unknown",Q24="Unknown"),"Needs date / judgment",IF(G24="Target","Target only","Pass")))</x:f>
-        <x:v>Needs date / judgment</x:v>
+        <x:f>IF(P24="After cutoff","Exclude: post-reference",IF(P24="Unknown","Needs observation date",IF(G24="Target","Target only","Observation-eligible")))</x:f>
+        <x:v>Observation-eligible</x:v>
       </x:c>
       <x:c r="S24" s="14" t="str">
-        <x:v>State industrial average, not a hyperscale contract price.</x:v>
+        <x:v>Preliminary calendar-2025 Texas industrial average: 6.55 cents/kWh. State industrial average, not a hyperscale contract price.</x:v>
       </x:c>
     </x:row>
     <x:row r="25">
@@ -2888,7 +2974,7 @@
         <x:v>Virginia</x:v>
       </x:c>
       <x:c r="E25" s="27" t="n">
-        <x:v>0.0899</x:v>
+        <x:v>0.0945</x:v>
       </x:c>
       <x:c r="F25" s="14" t="str">
         <x:v>USD/kWh</x:v>
@@ -2897,23 +2983,25 @@
         <x:v>Reported average</x:v>
       </x:c>
       <x:c r="H25" s="23" t="n">
-        <x:v>45657</x:v>
+        <x:v>46022</x:v>
       </x:c>
       <x:c r="I25" s="14" t="str">
         <x:v>Calendar year end</x:v>
       </x:c>
-      <x:c r="J25" s="23"/>
+      <x:c r="J25" s="23" t="n">
+        <x:v>46073</x:v>
+      </x:c>
       <x:c r="K25" s="14" t="str">
-        <x:v>Release day unrecorded</x:v>
+        <x:v>EIA preliminary release</x:v>
       </x:c>
       <x:c r="L25" s="14" t="str">
         <x:v>U.S. Energy Information Administration</x:v>
       </x:c>
       <x:c r="M25" s="14" t="str">
-        <x:v>Electric Power Annual table 2.10</x:v>
+        <x:v>Electric Power Monthly table 5.6.B</x:v>
       </x:c>
       <x:c r="N25" s="14" t="str">
-        <x:v>https://www.eia.gov/electricity/annual/table.php?t=epa_02_10.html</x:v>
+        <x:v>https://www.eia.gov/electricity/monthly/current_month/february2026.pdf</x:v>
       </x:c>
       <x:c r="O25" s="14" t="str">
         <x:v>Yes – chart height</x:v>
@@ -2924,14 +3012,14 @@
       </x:c>
       <x:c r="Q25" s="14" t="str">
         <x:f>IF(J25="","Unknown",IF(J25&lt;='Cutoff Policy'!$B$5,"Pass","After cutoff"))</x:f>
-        <x:v>Unknown</x:v>
+        <x:v>Pass</x:v>
       </x:c>
       <x:c r="R25" s="14" t="str">
-        <x:f>IF(OR(P25="After cutoff",Q25="After cutoff"),"Exclude from baseline",IF(OR(P25="Unknown",Q25="Unknown"),"Needs date / judgment",IF(G25="Target","Target only","Pass")))</x:f>
-        <x:v>Needs date / judgment</x:v>
+        <x:f>IF(P25="After cutoff","Exclude: post-reference",IF(P25="Unknown","Needs observation date",IF(G25="Target","Target only","Observation-eligible")))</x:f>
+        <x:v>Observation-eligible</x:v>
       </x:c>
       <x:c r="S25" s="14" t="str">
-        <x:v>State industrial average, not a hyperscale contract price.</x:v>
+        <x:v>Preliminary calendar-2025 Virginia industrial average: 9.45 cents/kWh. State industrial average, not a hyperscale contract price.</x:v>
       </x:c>
     </x:row>
     <x:row r="26">
@@ -2987,8 +3075,8 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="R26" s="14" t="str">
-        <x:f>IF(OR(P26="After cutoff",Q26="After cutoff"),"Exclude from baseline",IF(OR(P26="Unknown",Q26="Unknown"),"Needs date / judgment",IF(G26="Target","Target only","Pass")))</x:f>
-        <x:v>Needs date / judgment</x:v>
+        <x:f>IF(P26="After cutoff","Exclude: post-reference",IF(P26="Unknown","Needs observation date",IF(G26="Target","Target only","Observation-eligible")))</x:f>
+        <x:v>Observation-eligible</x:v>
       </x:c>
       <x:c r="S26" s="14" t="str">
         <x:v>Used for all China chart rows.</x:v>
@@ -3047,8 +3135,8 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="R27" s="14" t="str">
-        <x:f>IF(OR(P27="After cutoff",Q27="After cutoff"),"Exclude from baseline",IF(OR(P27="Unknown",Q27="Unknown"),"Needs date / judgment",IF(G27="Target","Target only","Pass")))</x:f>
-        <x:v>Needs date / judgment</x:v>
+        <x:f>IF(P27="After cutoff","Exclude: post-reference",IF(P27="Unknown","Needs observation date",IF(G27="Target","Target only","Observation-eligible")))</x:f>
+        <x:v>Observation-eligible</x:v>
       </x:c>
       <x:c r="S27" s="14" t="str">
         <x:v>Used for Montreal.</x:v>
@@ -3105,8 +3193,8 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="R28" s="14" t="str">
-        <x:f>IF(OR(P28="After cutoff",Q28="After cutoff"),"Exclude from baseline",IF(OR(P28="Unknown",Q28="Unknown"),"Needs date / judgment",IF(G28="Target","Target only","Pass")))</x:f>
-        <x:v>Needs date / judgment</x:v>
+        <x:f>IF(P28="After cutoff","Exclude: post-reference",IF(P28="Unknown","Needs observation date",IF(G28="Target","Target only","Observation-eligible")))</x:f>
+        <x:v>Needs observation date</x:v>
       </x:c>
       <x:c r="S28" s="14" t="str">
         <x:v>Fixed official parity; publication date is not stated.</x:v>
@@ -3163,8 +3251,8 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="R29" s="14" t="str">
-        <x:f>IF(OR(P29="After cutoff",Q29="After cutoff"),"Exclude from baseline",IF(OR(P29="Unknown",Q29="Unknown"),"Needs date / judgment",IF(G29="Target","Target only","Pass")))</x:f>
-        <x:v>Needs date / judgment</x:v>
+        <x:f>IF(P29="After cutoff","Exclude: post-reference",IF(P29="Unknown","Needs observation date",IF(G29="Target","Target only","Observation-eligible")))</x:f>
+        <x:v>Needs observation date</x:v>
       </x:c>
       <x:c r="S29" s="14" t="str">
         <x:v>Dense figure is half of the listed sparse BF16 value.</x:v>
@@ -3221,8 +3309,8 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="R30" s="14" t="str">
-        <x:f>IF(OR(P30="After cutoff",Q30="After cutoff"),"Exclude from baseline",IF(OR(P30="Unknown",Q30="Unknown"),"Needs date / judgment",IF(G30="Target","Target only","Pass")))</x:f>
-        <x:v>Needs date / judgment</x:v>
+        <x:f>IF(P30="After cutoff","Exclude: post-reference",IF(P30="Unknown","Needs observation date",IF(G30="Target","Target only","Observation-eligible")))</x:f>
+        <x:v>Needs observation date</x:v>
       </x:c>
       <x:c r="S30" s="14" t="str">
         <x:v>Full-load rack power including rack components; not a workload-metered result.</x:v>
@@ -3277,8 +3365,8 @@
         <x:v>Unknown</x:v>
       </x:c>
       <x:c r="R31" s="14" t="str">
-        <x:f>IF(OR(P31="After cutoff",Q31="After cutoff"),"Exclude from baseline",IF(OR(P31="Unknown",Q31="Unknown"),"Needs date / judgment",IF(G31="Target","Target only","Pass")))</x:f>
-        <x:v>Needs date / judgment</x:v>
+        <x:f>IF(P31="After cutoff","Exclude: post-reference",IF(P31="Unknown","Needs observation date",IF(G31="Target","Target only","Observation-eligible")))</x:f>
+        <x:v>Needs observation date</x:v>
       </x:c>
       <x:c r="S31" s="14" t="str">
         <x:v>Not an observed fact. Holding PUE fixed isolates electricity-price differences.</x:v>
@@ -3339,8 +3427,8 @@
         <x:v>Pass</x:v>
       </x:c>
       <x:c r="R32" s="14" t="str">
-        <x:f>IF(OR(P32="After cutoff",Q32="After cutoff"),"Exclude from baseline",IF(OR(P32="Unknown",Q32="Unknown"),"Needs date / judgment",IF(G32="Target","Target only","Pass")))</x:f>
-        <x:v>Pass</x:v>
+        <x:f>IF(P32="After cutoff","Exclude: post-reference",IF(P32="Unknown","Needs observation date",IF(G32="Target","Target only","Observation-eligible")))</x:f>
+        <x:v>Observation-eligible</x:v>
       </x:c>
       <x:c r="S32" s="14" t="str">
         <x:v>Direct later observation; not substituted because the baseline provincial series uses a common March boundary.</x:v>
@@ -3401,8 +3489,8 @@
         <x:v>Pass</x:v>
       </x:c>
       <x:c r="R33" s="14" t="str">
-        <x:f>IF(OR(P33="After cutoff",Q33="After cutoff"),"Exclude from baseline",IF(OR(P33="Unknown",Q33="Unknown"),"Needs date / judgment",IF(G33="Target","Target only","Pass")))</x:f>
-        <x:v>Pass</x:v>
+        <x:f>IF(P33="After cutoff","Exclude: post-reference",IF(P33="Unknown","Needs observation date",IF(G33="Target","Target only","Observation-eligible")))</x:f>
+        <x:v>Observation-eligible</x:v>
       </x:c>
       <x:c r="S33" s="14" t="str">
         <x:v>Total capacity boundary; may not equal CAICT in-use design racks.</x:v>
@@ -3463,8 +3551,8 @@
         <x:v>Pass</x:v>
       </x:c>
       <x:c r="R34" s="14" t="str">
-        <x:f>IF(OR(P34="After cutoff",Q34="After cutoff"),"Exclude from baseline",IF(OR(P34="Unknown",Q34="Unknown"),"Needs date / judgment",IF(G34="Target","Target only","Pass")))</x:f>
-        <x:v>Pass</x:v>
+        <x:f>IF(P34="After cutoff","Exclude: post-reference",IF(P34="Unknown","Needs observation date",IF(G34="Target","Target only","Observation-eligible")))</x:f>
+        <x:v>Observation-eligible</x:v>
       </x:c>
       <x:c r="S34" s="14" t="str">
         <x:v>Direct later observation.</x:v>
@@ -3525,8 +3613,8 @@
         <x:v>Pass</x:v>
       </x:c>
       <x:c r="R35" s="14" t="str">
-        <x:f>IF(OR(P35="After cutoff",Q35="After cutoff"),"Exclude from baseline",IF(OR(P35="Unknown",Q35="Unknown"),"Needs date / judgment",IF(G35="Target","Target only","Pass")))</x:f>
-        <x:v>Pass</x:v>
+        <x:f>IF(P35="After cutoff","Exclude: post-reference",IF(P35="Unknown","Needs observation date",IF(G35="Target","Target only","Observation-eligible")))</x:f>
+        <x:v>Observation-eligible</x:v>
       </x:c>
       <x:c r="S35" s="14" t="str">
         <x:v>Built-rack boundary, not necessarily in-use design racks.</x:v>
@@ -3587,8 +3675,8 @@
         <x:v>Pass</x:v>
       </x:c>
       <x:c r="R36" s="14" t="str">
-        <x:f>IF(OR(P36="After cutoff",Q36="After cutoff"),"Exclude from baseline",IF(OR(P36="Unknown",Q36="Unknown"),"Needs date / judgment",IF(G36="Target","Target only","Pass")))</x:f>
-        <x:v>Pass</x:v>
+        <x:f>IF(P36="After cutoff","Exclude: post-reference",IF(P36="Unknown","Needs observation date",IF(G36="Target","Target only","Observation-eligible")))</x:f>
+        <x:v>Observation-eligible</x:v>
       </x:c>
       <x:c r="S36" s="14" t="str">
         <x:v>As-of wording is 'currently'; publication date used as observation-date proxy.</x:v>
@@ -3649,8 +3737,8 @@
         <x:v>Pass</x:v>
       </x:c>
       <x:c r="R37" s="14" t="str">
-        <x:f>IF(OR(P37="After cutoff",Q37="After cutoff"),"Exclude from baseline",IF(OR(P37="Unknown",Q37="Unknown"),"Needs date / judgment",IF(G37="Target","Target only","Pass")))</x:f>
-        <x:v>Pass</x:v>
+        <x:f>IF(P37="After cutoff","Exclude: post-reference",IF(P37="Unknown","Needs observation date",IF(G37="Target","Target only","Observation-eligible")))</x:f>
+        <x:v>Observation-eligible</x:v>
       </x:c>
       <x:c r="S37" s="14" t="str">
         <x:v>Direct later observation.</x:v>
@@ -3711,8 +3799,8 @@
         <x:v>Pass</x:v>
       </x:c>
       <x:c r="R38" s="14" t="str">
-        <x:f>IF(OR(P38="After cutoff",Q38="After cutoff"),"Exclude from baseline",IF(OR(P38="Unknown",Q38="Unknown"),"Needs date / judgment",IF(G38="Target","Target only","Pass")))</x:f>
-        <x:v>Pass</x:v>
+        <x:f>IF(P38="After cutoff","Exclude: post-reference",IF(P38="Unknown","Needs observation date",IF(G38="Target","Target only","Observation-eligible")))</x:f>
+        <x:v>Observation-eligible</x:v>
       </x:c>
       <x:c r="S38" s="14" t="str">
         <x:v>Boundary covers 50 centres under construction or in operation; not comparable to in-use racks.</x:v>
@@ -3773,8 +3861,8 @@
         <x:v>Pass</x:v>
       </x:c>
       <x:c r="R39" s="14" t="str">
-        <x:f>IF(OR(P39="After cutoff",Q39="After cutoff"),"Exclude from baseline",IF(OR(P39="Unknown",Q39="Unknown"),"Needs date / judgment",IF(G39="Target","Target only","Pass")))</x:f>
-        <x:v>Pass</x:v>
+        <x:f>IF(P39="After cutoff","Exclude: post-reference",IF(P39="Unknown","Needs observation date",IF(G39="Target","Target only","Observation-eligible")))</x:f>
+        <x:v>Observation-eligible</x:v>
       </x:c>
       <x:c r="S39" s="14" t="str">
         <x:v>Government-page mirror; source authenticity should be rechecked.</x:v>
@@ -3835,8 +3923,8 @@
         <x:v>Pass</x:v>
       </x:c>
       <x:c r="R40" s="14" t="str">
-        <x:f>IF(OR(P40="After cutoff",Q40="After cutoff"),"Exclude from baseline",IF(OR(P40="Unknown",Q40="Unknown"),"Needs date / judgment",IF(G40="Target","Target only","Pass")))</x:f>
-        <x:v>Pass</x:v>
+        <x:f>IF(P40="After cutoff","Exclude: post-reference",IF(P40="Unknown","Needs observation date",IF(G40="Target","Target only","Observation-eligible")))</x:f>
+        <x:v>Observation-eligible</x:v>
       </x:c>
       <x:c r="S40" s="14" t="str">
         <x:v>Government-page mirror; rack standardisation is not clear.</x:v>
@@ -3897,8 +3985,8 @@
         <x:v>Pass</x:v>
       </x:c>
       <x:c r="R41" s="14" t="str">
-        <x:f>IF(OR(P41="After cutoff",Q41="After cutoff"),"Exclude from baseline",IF(OR(P41="Unknown",Q41="Unknown"),"Needs date / judgment",IF(G41="Target","Target only","Pass")))</x:f>
-        <x:v>Pass</x:v>
+        <x:f>IF(P41="After cutoff","Exclude: post-reference",IF(P41="Unknown","Needs observation date",IF(G41="Target","Target only","Observation-eligible")))</x:f>
+        <x:v>Observation-eligible</x:v>
       </x:c>
       <x:c r="S41" s="14" t="str">
         <x:v>Secondary article quoting the regulator.</x:v>
@@ -3959,8 +4047,8 @@
         <x:v>Pass</x:v>
       </x:c>
       <x:c r="R42" s="14" t="str">
-        <x:f>IF(OR(P42="After cutoff",Q42="After cutoff"),"Exclude from baseline",IF(OR(P42="Unknown",Q42="Unknown"),"Needs date / judgment",IF(G42="Target","Target only","Pass")))</x:f>
-        <x:v>Pass</x:v>
+        <x:f>IF(P42="After cutoff","Exclude: post-reference",IF(P42="Unknown","Needs observation date",IF(G42="Target","Target only","Observation-eligible")))</x:f>
+        <x:v>Observation-eligible</x:v>
       </x:c>
       <x:c r="S42" s="14" t="str">
         <x:v>Secondary article quoting the regulator.</x:v>
@@ -4021,8 +4109,8 @@
         <x:v>Pass</x:v>
       </x:c>
       <x:c r="R43" s="14" t="str">
-        <x:f>IF(OR(P43="After cutoff",Q43="After cutoff"),"Exclude from baseline",IF(OR(P43="Unknown",Q43="Unknown"),"Needs date / judgment",IF(G43="Target","Target only","Pass")))</x:f>
-        <x:v>Pass</x:v>
+        <x:f>IF(P43="After cutoff","Exclude: post-reference",IF(P43="Unknown","Needs observation date",IF(G43="Target","Target only","Observation-eligible")))</x:f>
+        <x:v>Observation-eligible</x:v>
       </x:c>
       <x:c r="S43" s="14" t="str">
         <x:v>Commercial IDC cabinets, not CAICT-standardised racks.</x:v>
@@ -4083,8 +4171,8 @@
         <x:v>Pass</x:v>
       </x:c>
       <x:c r="R44" s="14" t="str">
-        <x:f>IF(OR(P44="After cutoff",Q44="After cutoff"),"Exclude from baseline",IF(OR(P44="Unknown",Q44="Unknown"),"Needs date / judgment",IF(G44="Target","Target only","Pass")))</x:f>
-        <x:v>Pass</x:v>
+        <x:f>IF(P44="After cutoff","Exclude: post-reference",IF(P44="Unknown","Needs observation date",IF(G44="Target","Target only","Observation-eligible")))</x:f>
+        <x:v>Observation-eligible</x:v>
       </x:c>
       <x:c r="S44" s="14" t="str">
         <x:v>Secondary disclosure citing CAICT; standard-rack basis not stated in the article.</x:v>
@@ -4145,8 +4233,8 @@
         <x:v>Pass</x:v>
       </x:c>
       <x:c r="R45" s="14" t="str">
-        <x:f>IF(OR(P45="After cutoff",Q45="After cutoff"),"Exclude from baseline",IF(OR(P45="Unknown",Q45="Unknown"),"Needs date / judgment",IF(G45="Target","Target only","Pass")))</x:f>
-        <x:v>Pass</x:v>
+        <x:f>IF(P45="After cutoff","Exclude: post-reference",IF(P45="Unknown","Needs observation date",IF(G45="Target","Target only","Observation-eligible")))</x:f>
+        <x:v>Observation-eligible</x:v>
       </x:c>
       <x:c r="S45" s="14" t="str">
         <x:v>Article says more than 350,000; register stores 350,000 as a lower bound.</x:v>

</xml_diff>

<commit_message>
fix: use applicable Montreal electricity tariff
</commit_message>
<xml_diff>
--- a/outputs/019fdb9f-161f-7b22-9a01-b1a28036fbf3/capacity-source-register.xlsx
+++ b/outputs/019fdb9f-161f-7b22-9a01-b1a28036fbf3/capacity-source-register.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cutoff Policy" sheetId="1" r:id="Rcb98fe5ae625438c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Curve Inputs" sheetId="2" r:id="Rae4c2eb312224165"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Register" sheetId="3" r:id="R39c3b30f53ba45cf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cutoff Policy" sheetId="1" r:id="R10afe41f56c94cf8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Curve Inputs" sheetId="2" r:id="R6e2666be1ddb4e5a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Register" sheetId="3" r:id="R72bbd809f2dd430f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -15,11 +15,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="4">
+  <x:numFmts count="5">
     <x:numFmt numFmtId="200" formatCode="yyyy-mm-dd"/>
     <x:numFmt numFmtId="201" formatCode="0.0"/>
     <x:numFmt numFmtId="202" formatCode="0.0000000"/>
     <x:numFmt numFmtId="203" formatCode="0.########"/>
+    <x:numFmt numFmtId="204" formatCode="0%"/>
   </x:numFmts>
   <x:fonts count="5">
     <x:font>
@@ -94,7 +95,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="34">
+  <x:cellXfs count="36">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -170,6 +171,10 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="204" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -1418,10 +1423,11 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="H17" s="24" t="n">
-        <x:v>0.0375438</x:v>
+        <x:f>'Source Register'!E22/'Source Register'!E27</x:f>
+        <x:v>0.043921136882709544</x:v>
       </x:c>
       <x:c r="I17" s="23" t="n">
-        <x:v>46022</x:v>
+        <x:v>45748</x:v>
       </x:c>
       <x:c r="J17" s="23"/>
       <x:c r="K17" s="14" t="str">
@@ -1448,7 +1454,7 @@
         <x:v>https://www.cbre.com/press-releases/northern-virginia-extends-lead-as-largest-u-s-data-center-market-in-2025</x:v>
       </x:c>
       <x:c r="Q17" s="14" t="str">
-        <x:v>https://www.hydroquebec.com/data/documents-donnees/pdf/rates-chart-2025.pdf — Wholesale H2 2025 market inventory; Rate L effective price. Rate-chart publication day is unrecorded.</x:v>
+        <x:v>https://www.hydroquebec.com/data/documents-donnees/pdf/electricity-rates.pdf?v=HT-2025-v3 — Wholesale H2 2025 market inventory; applicable Rate LG proxy at 120 kV and 90% load factor. Hydro-Québec's 2026 filing identifies 2025 data centres as Rate M or LG customers: https://www.regie-energie.qc.ca/fr/participants/dossiers/R-4333-2026/doc/R-4333-2026-B-0004-Dem-Piece-2026_02_19.pdf</x:v>
       </x:c>
       <x:c r="R17" s="14" t="str">
         <x:v>Included</x:v>
@@ -2788,38 +2794,39 @@
         <x:v>Electricity price</x:v>
       </x:c>
       <x:c r="C22" s="14" t="str">
-        <x:v>Quebec Rate L effective price</x:v>
+        <x:v>Quebec Rate LG tariff proxy</x:v>
       </x:c>
       <x:c r="D22" s="14" t="str">
         <x:v>Quebec</x:v>
       </x:c>
       <x:c r="E22" s="27" t="n">
-        <x:v>0.05246</x:v>
+        <x:f>E46+(E47-E48)/(E49*E50)</x:f>
+        <x:v>0.061371004566210044</x:v>
       </x:c>
       <x:c r="F22" s="14" t="str">
         <x:v>CAD/kWh</x:v>
       </x:c>
       <x:c r="G22" s="14" t="str">
-        <x:v>Derived from tariff</x:v>
+        <x:v>Derived from applicable tariff</x:v>
       </x:c>
       <x:c r="H22" s="23" t="n">
-        <x:v>46022</x:v>
+        <x:v>45748</x:v>
       </x:c>
       <x:c r="I22" s="14" t="str">
-        <x:v>2025 rate year</x:v>
+        <x:v>Exact effective day</x:v>
       </x:c>
       <x:c r="J22" s="23"/>
       <x:c r="K22" s="14" t="str">
-        <x:v>Unrecorded</x:v>
+        <x:v>Official tariff effective 2025-04-01</x:v>
       </x:c>
       <x:c r="L22" s="14" t="str">
         <x:v>Hydro-Québec</x:v>
       </x:c>
       <x:c r="M22" s="14" t="str">
-        <x:v>Rate chart 2025</x:v>
+        <x:v>Electricity Rates Effective April 1, 2025</x:v>
       </x:c>
       <x:c r="N22" s="14" t="str">
-        <x:v>https://www.hydroquebec.com/data/documents-donnees/pdf/rates-chart-2025.pdf</x:v>
+        <x:v>https://www.hydroquebec.com/data/documents-donnees/pdf/electricity-rates.pdf?v=HT-2025-v3</x:v>
       </x:c>
       <x:c r="O22" s="14" t="str">
         <x:v>Yes – chart height</x:v>
@@ -2837,7 +2844,7 @@
         <x:v>Observation-eligible</x:v>
       </x:c>
       <x:c r="S22" s="14" t="str">
-        <x:v>Effective price at 120 kV and 100% load factor.</x:v>
+        <x:v>Rate LG applies to non-industrial large-power data centres. Proxy at 120 kV and 90% load factor: CAD 0.04165/kWh + (CAD 15.963 − CAD 3.0063)/(730 h × 90%) = CAD 0.0613711/kWh. Applicability cross-check: https://www.regie-energie.qc.ca/fr/participants/dossiers/R-4333-2026/doc/R-4333-2026-B-0004-Dem-Piece-2026_02_19.pdf</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
@@ -3139,7 +3146,7 @@
         <x:v>Observation-eligible</x:v>
       </x:c>
       <x:c r="S27" s="14" t="str">
-        <x:v>Used for Montreal.</x:v>
+        <x:v>Used to convert Montreal's Rate LG tariff proxy from CAD to USD.</x:v>
       </x:c>
     </x:row>
     <x:row r="28">
@@ -4238,6 +4245,283 @@
       </x:c>
       <x:c r="S45" s="14" t="str">
         <x:v>Article says more than 350,000; register stores 350,000 as a lower bound.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" ht="34" customHeight="1">
+      <x:c r="A46" s="13" t="str">
+        <x:v>SRC-043</x:v>
+      </x:c>
+      <x:c r="B46" s="13" t="str">
+        <x:v>Electricity price</x:v>
+      </x:c>
+      <x:c r="C46" s="13" t="str">
+        <x:v>Quebec Rate LG energy charge</x:v>
+      </x:c>
+      <x:c r="D46" s="13" t="str">
+        <x:v>Quebec</x:v>
+      </x:c>
+      <x:c r="E46" s="13" t="n">
+        <x:v>0.04165</x:v>
+      </x:c>
+      <x:c r="F46" s="13" t="str">
+        <x:v>CAD/kWh</x:v>
+      </x:c>
+      <x:c r="G46" s="13" t="str">
+        <x:v>Published tariff</x:v>
+      </x:c>
+      <x:c r="H46" s="20" t="n">
+        <x:v>45748</x:v>
+      </x:c>
+      <x:c r="I46" s="13" t="str">
+        <x:v>Exact effective day</x:v>
+      </x:c>
+      <x:c r="J46" s="13"/>
+      <x:c r="K46" s="13" t="str">
+        <x:v>Official tariff effective 2025-04-01</x:v>
+      </x:c>
+      <x:c r="L46" s="13" t="str">
+        <x:v>Hydro-Québec</x:v>
+      </x:c>
+      <x:c r="M46" s="13" t="str">
+        <x:v>Electricity Rates Effective April 1, 2025</x:v>
+      </x:c>
+      <x:c r="N46" s="13" t="str">
+        <x:v>https://www.hydroquebec.com/data/documents-donnees/pdf/electricity-rates.pdf?v=HT-2025-v3</x:v>
+      </x:c>
+      <x:c r="O46" s="13" t="str">
+        <x:v>Yes – tariff formula</x:v>
+      </x:c>
+      <x:c r="P46" s="13" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="Q46" s="13" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="R46" s="13" t="str">
+        <x:v>Observation-eligible</x:v>
+      </x:c>
+      <x:c r="S46" s="13" t="str">
+        <x:v>Rate LG energy component for non-industrial large-power contracts.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47" ht="34" customHeight="1">
+      <x:c r="A47" s="13" t="str">
+        <x:v>SRC-044</x:v>
+      </x:c>
+      <x:c r="B47" s="13" t="str">
+        <x:v>Electricity price</x:v>
+      </x:c>
+      <x:c r="C47" s="13" t="str">
+        <x:v>Quebec Rate LG demand charge</x:v>
+      </x:c>
+      <x:c r="D47" s="13" t="str">
+        <x:v>Quebec</x:v>
+      </x:c>
+      <x:c r="E47" s="13" t="n">
+        <x:v>15.963</x:v>
+      </x:c>
+      <x:c r="F47" s="13" t="str">
+        <x:v>CAD/kW-month</x:v>
+      </x:c>
+      <x:c r="G47" s="13" t="str">
+        <x:v>Published tariff</x:v>
+      </x:c>
+      <x:c r="H47" s="20" t="n">
+        <x:v>45748</x:v>
+      </x:c>
+      <x:c r="I47" s="13" t="str">
+        <x:v>Exact effective day</x:v>
+      </x:c>
+      <x:c r="J47" s="13"/>
+      <x:c r="K47" s="13" t="str">
+        <x:v>Official tariff effective 2025-04-01</x:v>
+      </x:c>
+      <x:c r="L47" s="13" t="str">
+        <x:v>Hydro-Québec</x:v>
+      </x:c>
+      <x:c r="M47" s="13" t="str">
+        <x:v>Electricity Rates Effective April 1, 2025</x:v>
+      </x:c>
+      <x:c r="N47" s="13" t="str">
+        <x:v>https://www.hydroquebec.com/data/documents-donnees/pdf/electricity-rates.pdf?v=HT-2025-v3</x:v>
+      </x:c>
+      <x:c r="O47" s="13" t="str">
+        <x:v>Yes – tariff formula</x:v>
+      </x:c>
+      <x:c r="P47" s="13" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="Q47" s="13" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="R47" s="13" t="str">
+        <x:v>Observation-eligible</x:v>
+      </x:c>
+      <x:c r="S47" s="13" t="str">
+        <x:v>Monthly Rate LG demand charge.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48" ht="34" customHeight="1">
+      <x:c r="A48" s="13" t="str">
+        <x:v>SRC-045</x:v>
+      </x:c>
+      <x:c r="B48" s="13" t="str">
+        <x:v>Electricity price</x:v>
+      </x:c>
+      <x:c r="C48" s="13" t="str">
+        <x:v>Quebec 120 kV high-voltage supply credit</x:v>
+      </x:c>
+      <x:c r="D48" s="13" t="str">
+        <x:v>Quebec</x:v>
+      </x:c>
+      <x:c r="E48" s="13" t="n">
+        <x:v>3.0063</x:v>
+      </x:c>
+      <x:c r="F48" s="13" t="str">
+        <x:v>CAD/kW-month</x:v>
+      </x:c>
+      <x:c r="G48" s="13" t="str">
+        <x:v>Published tariff</x:v>
+      </x:c>
+      <x:c r="H48" s="20" t="n">
+        <x:v>45748</x:v>
+      </x:c>
+      <x:c r="I48" s="13" t="str">
+        <x:v>Exact effective day</x:v>
+      </x:c>
+      <x:c r="J48" s="13"/>
+      <x:c r="K48" s="13" t="str">
+        <x:v>Official tariff effective 2025-04-01</x:v>
+      </x:c>
+      <x:c r="L48" s="13" t="str">
+        <x:v>Hydro-Québec</x:v>
+      </x:c>
+      <x:c r="M48" s="13" t="str">
+        <x:v>Electricity Rates Effective April 1, 2025</x:v>
+      </x:c>
+      <x:c r="N48" s="13" t="str">
+        <x:v>https://www.hydroquebec.com/data/documents-donnees/pdf/electricity-rates.pdf?v=HT-2025-v3</x:v>
+      </x:c>
+      <x:c r="O48" s="13" t="str">
+        <x:v>Yes – tariff formula</x:v>
+      </x:c>
+      <x:c r="P48" s="13" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="Q48" s="13" t="str">
+        <x:v>Unknown</x:v>
+      </x:c>
+      <x:c r="R48" s="13" t="str">
+        <x:v>Observation-eligible</x:v>
+      </x:c>
+      <x:c r="S48" s="13" t="str">
+        <x:v>Credit for supply at 80 kV or more but less than 170 kV; 120 kV is within this band.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" ht="34" customHeight="1">
+      <x:c r="A49" s="13" t="str">
+        <x:v>SRC-046</x:v>
+      </x:c>
+      <x:c r="B49" s="13" t="str">
+        <x:v>Method assumption</x:v>
+      </x:c>
+      <x:c r="C49" s="13" t="str">
+        <x:v>Montreal tariff-proxy load factor</x:v>
+      </x:c>
+      <x:c r="D49" s="13" t="str">
+        <x:v>Quebec</x:v>
+      </x:c>
+      <x:c r="E49" s="35" t="n">
+        <x:v>0.9</x:v>
+      </x:c>
+      <x:c r="F49" s="13" t="str">
+        <x:v>ratio</x:v>
+      </x:c>
+      <x:c r="G49" s="13" t="str">
+        <x:v>Analytical assumption</x:v>
+      </x:c>
+      <x:c r="H49" s="13"/>
+      <x:c r="I49" s="13" t="str">
+        <x:v>Not applicable</x:v>
+      </x:c>
+      <x:c r="J49" s="13"/>
+      <x:c r="K49" s="13" t="str">
+        <x:v>Not applicable</x:v>
+      </x:c>
+      <x:c r="L49" s="13" t="str">
+        <x:v>Project assumption</x:v>
+      </x:c>
+      <x:c r="M49" s="13" t="str">
+        <x:v>Common tariff-proxy convention</x:v>
+      </x:c>
+      <x:c r="N49" s="13" t="str"/>
+      <x:c r="O49" s="13" t="str">
+        <x:v>Yes – tariff formula</x:v>
+      </x:c>
+      <x:c r="P49" s="13" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="Q49" s="13" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="R49" s="13" t="str">
+        <x:v>Analytical assumption</x:v>
+      </x:c>
+      <x:c r="S49" s="13" t="str">
+        <x:v>Same 90% load-factor convention used for the Chinese two-part tariff proxies.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50" ht="34" customHeight="1">
+      <x:c r="A50" s="13" t="str">
+        <x:v>SRC-047</x:v>
+      </x:c>
+      <x:c r="B50" s="13" t="str">
+        <x:v>Method assumption</x:v>
+      </x:c>
+      <x:c r="C50" s="13" t="str">
+        <x:v>Hours per average billing month</x:v>
+      </x:c>
+      <x:c r="D50" s="13" t="str">
+        <x:v>Global tariff proxies</x:v>
+      </x:c>
+      <x:c r="E50" s="13" t="n">
+        <x:v>730</x:v>
+      </x:c>
+      <x:c r="F50" s="13" t="str">
+        <x:v>hours/month</x:v>
+      </x:c>
+      <x:c r="G50" s="13" t="str">
+        <x:v>Analytical convention</x:v>
+      </x:c>
+      <x:c r="H50" s="13"/>
+      <x:c r="I50" s="13" t="str">
+        <x:v>Not applicable</x:v>
+      </x:c>
+      <x:c r="J50" s="13"/>
+      <x:c r="K50" s="13" t="str">
+        <x:v>Not applicable</x:v>
+      </x:c>
+      <x:c r="L50" s="13" t="str">
+        <x:v>Project assumption</x:v>
+      </x:c>
+      <x:c r="M50" s="13" t="str">
+        <x:v>Common tariff-proxy convention</x:v>
+      </x:c>
+      <x:c r="N50" s="13" t="str"/>
+      <x:c r="O50" s="13" t="str">
+        <x:v>Yes – tariff formula</x:v>
+      </x:c>
+      <x:c r="P50" s="13" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="Q50" s="13" t="str">
+        <x:v>Pass</x:v>
+      </x:c>
+      <x:c r="R50" s="13" t="str">
+        <x:v>Analytical assumption</x:v>
+      </x:c>
+      <x:c r="S50" s="13" t="str">
+        <x:v>Used to convert monthly demand charges to per-kWh equivalents.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>